<commit_message>
scan: seg5 2026-06-19 15:03 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-06-18.xlsx
+++ b/output/full_scan/batch_seq7_2026-06-18.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O79"/>
+  <dimension ref="A1:O80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2700,21 +2700,21 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6570</v>
+        <v>6727</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>維田</t>
+          <t>亞泰金屬</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>496.1486317061344</v>
+        <v>503.4645960592337</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>54.6</v>
+        <v>449</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,16 +2725,16 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>52.42481175718345</v>
+        <v>47.52615106428384</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>23.76705450469684</v>
+        <v>20.89367945259401</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.3833070275867184</v>
+        <v>0.6727984200975592</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-1.109068786778863</v>
+        <v>-13.08914703597903</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6581</v>
+        <v>6570</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>鋼聯</t>
+          <t>維田</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>479.970592358576</v>
+        <v>496.1486317061344</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>109</v>
+        <v>54.6</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>51.89955966305028</v>
+        <v>52.42481175718345</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>12.11252179967143</v>
+        <v>23.76705450469684</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.3768419376858822</v>
+        <v>0.3833070275867184</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.0665971308961273</v>
+        <v>-1.109068786778863</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6669</v>
+        <v>6581</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>緯穎</t>
+          <t>鋼聯</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>466.1181689692934</v>
+        <v>479.970592358576</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>5130</v>
+        <v>109</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,16 +2831,16 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>50.88120539285397</v>
+        <v>51.89955966305028</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>18.14533992693503</v>
+        <v>12.11252179967143</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.8772528763705716</v>
+        <v>0.3768419376858822</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-67.9570811290519</v>
+        <v>-0.0665971308961273</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6679</v>
+        <v>6669</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>鈺太</t>
+          <t>緯穎</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>453.6898377236356</v>
+        <v>466.1181689692934</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>285.5</v>
+        <v>5130</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,16 +2884,16 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>48.85136040216892</v>
+        <v>50.88120539285397</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>23.89648805720262</v>
+        <v>18.14533992693503</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>1.11668301656967</v>
+        <v>0.8772528763705716</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-2.101179549021317</v>
+        <v>-67.9570811290519</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6664</v>
+        <v>6679</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>群翊</t>
+          <t>鈺太</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>449.3570211672675</v>
+        <v>453.6898377236356</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>384.5</v>
+        <v>285.5</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,49 +2937,49 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>43.94022319526404</v>
+        <v>48.85136040216892</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>25.01642423037803</v>
+        <v>23.89648805720262</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.4493816809447752</v>
+        <v>1.11668301656967</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-3.31959791684152</v>
+        <v>-2.101179549021317</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, dealer_buy_3d</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6597</v>
+        <v>6664</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>立誠</t>
+          <t>群翊</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>440.8706393226338</v>
+        <v>449.3570211672675</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>69.90000000000001</v>
+        <v>384.5</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,49 +2990,49 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>50.3642279826005</v>
+        <v>43.94022319526404</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>10.95342029530177</v>
+        <v>25.01642423037803</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.3987806652451872</v>
+        <v>0.4493816809447752</v>
       </c>
       <c r="K48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L48" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M48" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.8235082161255737</v>
+        <v>-3.31959791684152</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6640</v>
+        <v>6597</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>均華</t>
+          <t>立誠</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>421.0881588648485</v>
+        <v>440.8706393226338</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>1120</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,49 +3043,49 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>40.2277505211943</v>
+        <v>50.3642279826005</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>26.20414624338033</v>
+        <v>10.95342029530177</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.6745921331383645</v>
+        <v>0.3987806652451872</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M49" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-5.844428668762077</v>
+        <v>-0.8235082161255737</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6776</v>
+        <v>6640</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>展碁國際</t>
+          <t>均華</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>413.0446299831584</v>
+        <v>421.0881588648485</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>59.3</v>
+        <v>1120</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,49 +3096,49 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>49.98653859611562</v>
+        <v>40.2277505211943</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>9.190569822775885</v>
+        <v>26.20414624338033</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.7364648797195718</v>
+        <v>0.6745921331383645</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M50" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.1373214024441919</v>
+        <v>-5.844428668762077</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6588</v>
+        <v>6776</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>東典光電</t>
+          <t>展碁國際</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>407.8954663890353</v>
+        <v>413.0446299831584</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>107.5</v>
+        <v>59.3</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>42.35619710147279</v>
+        <v>49.98653859611562</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>16.27212687535586</v>
+        <v>9.190569822775885</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.4403768233267193</v>
+        <v>0.7364648797195718</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.6431512648268365</v>
+        <v>-0.1373214024441919</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6805</v>
+        <v>6588</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>富世達</t>
+          <t>東典光電</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>398.7284014102837</v>
+        <v>407.8954663890353</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>1755</v>
+        <v>107.5</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,16 +3202,16 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>44.56001974637073</v>
+        <v>42.35619710147279</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>14.95563451346673</v>
+        <v>16.27212687535586</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.4235421821256706</v>
+        <v>0.4403768233267193</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-22.32059347337242</v>
+        <v>0.6431512648268365</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6584</v>
+        <v>6805</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>南俊國際</t>
+          <t>富世達</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>392.2995944331854</v>
+        <v>398.7284014102837</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>625</v>
+        <v>1755</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>47.24033082115122</v>
+        <v>44.56001974637073</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>11.99895627351633</v>
+        <v>14.95563451346673</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.4166067427830628</v>
+        <v>0.4235421821256706</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-4.897651497646235</v>
+        <v>-22.32059347337242</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6720</v>
+        <v>6584</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>久昌</t>
+          <t>南俊國際</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>367.5597018916417</v>
+        <v>392.2995944331854</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>142</v>
+        <v>625</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>31.40520770213884</v>
+        <v>47.24033082115122</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>32.37499213641874</v>
+        <v>11.99895627351633</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.4962433826211615</v>
+        <v>0.4166067427830628</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.4338529336626631</v>
+        <v>-4.897651497646235</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6560</v>
+        <v>6720</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>欣普羅</t>
+          <t>久昌</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>365.8166742834656</v>
+        <v>367.5597018916417</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>38</v>
+        <v>142</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>48.66411407423659</v>
+        <v>31.40520770213884</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>13.89738325434931</v>
+        <v>32.37499213641874</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.4769321523662099</v>
+        <v>0.4962433826211615</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>2</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.1219414082608044</v>
+        <v>-0.4338529336626631</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6532</v>
+        <v>6560</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>瑞耘</t>
+          <t>欣普羅</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>357.8915831923025</v>
+        <v>365.8166742834656</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>91.2</v>
+        <v>38</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>46.09019394034403</v>
+        <v>48.66411407423659</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>22.77687482106036</v>
+        <v>13.89738325434931</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.4693127005229541</v>
+        <v>0.4769321523662099</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>2</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.9849691377950304</v>
+        <v>-0.1219414082608044</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6512</v>
+        <v>6532</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>啟發電</t>
+          <t>瑞耘</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>350.8206024752992</v>
+        <v>357.8915831923025</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>19.5</v>
+        <v>91.2</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,16 +3467,16 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>51.80891999353064</v>
+        <v>46.09019394034403</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>9.097562983992548</v>
+        <v>22.77687482106036</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.5410566937326722</v>
+        <v>0.4693127005229541</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.3545710958930965</v>
+        <v>-0.9849691377950304</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6771</v>
+        <v>6512</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>平和環保-創</t>
+          <t>啟發電</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>344.8325442287269</v>
+        <v>350.8206024752992</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>42</v>
+        <v>19.5</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>46.22371642440847</v>
+        <v>51.80891999353064</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>14.02746498428115</v>
+        <v>9.097562983992548</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>2.296825479077181</v>
+        <v>0.5410566937326722</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.0948303683630313</v>
+        <v>-0.3545710958930965</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6743</v>
+        <v>6771</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>安普新</t>
+          <t>平和環保-創</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>338.3828257707834</v>
+        <v>344.8325442287269</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>49.50494794959324</v>
+        <v>46.22371642440847</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>19.60396743861664</v>
+        <v>14.02746498428115</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.4233598211674846</v>
+        <v>2.296825479077181</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.2274145851520772</v>
+        <v>0.0948303683630313</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6692</v>
+        <v>6743</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>進能服</t>
+          <t>安普新</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>337.5501471522792</v>
+        <v>338.3828257707834</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>48.54069699700314</v>
+        <v>49.50494794959324</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>22.41233210320248</v>
+        <v>19.60396743861664</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>1.334770468634914</v>
+        <v>0.4233598211674846</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.2841797902961656</v>
+        <v>-0.2274145851520772</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, stronger_than_market, obv_uptrend</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6708</v>
+        <v>6692</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>天擎</t>
+          <t>進能服</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>331.1617641552466</v>
+        <v>337.5501471522792</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>39.8</v>
+        <v>27</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,16 +3679,16 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>47.69413375504143</v>
+        <v>48.54069699700314</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>15.1933117230612</v>
+        <v>22.41233210320248</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.513416997832753</v>
+        <v>1.334770468634914</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.0563190215787685</v>
+        <v>0.2841797902961656</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend</t>
+          <t>market_above_ma60, adx_trending, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6643</v>
+        <v>6708</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>M31</t>
+          <t>天擎</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>326.7879391794831</v>
+        <v>331.1617641552466</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>494</v>
+        <v>39.8</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>40.73448371625519</v>
+        <v>47.69413375504143</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>26.40102873469428</v>
+        <v>15.1933117230612</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.598897058187882</v>
+        <v>0.513416997832753</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-6.037609793522932</v>
+        <v>-0.0563190215787685</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6806</v>
+        <v>6643</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>森崴能源</t>
+          <t>M31</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>321.1806280133556</v>
+        <v>326.7879391794831</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>3.24</v>
+        <v>494</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>30.30810162010731</v>
+        <v>40.73448371625519</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>32.28363367198867</v>
+        <v>26.40102873469428</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>1.437623507568395</v>
+        <v>0.598897058187882</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.3767060656906009</v>
+        <v>-6.037609793522932</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6706</v>
+        <v>6806</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>惠特</t>
+          <t>森崴能源</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>319.8451855910437</v>
+        <v>321.1806280133556</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>172</v>
+        <v>3.24</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>48.69595574494014</v>
+        <v>30.30810162010731</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>18.33759879254464</v>
+        <v>32.28363367198867</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.4565582620914242</v>
+        <v>1.437623507568395</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-3.936865684636677</v>
+        <v>0.3767060656906009</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6546</v>
+        <v>6706</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>正基</t>
+          <t>惠特</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>312.9547032703164</v>
+        <v>319.8451855910437</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>75</v>
+        <v>172</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,16 +3891,16 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>50.17604797029433</v>
+        <v>48.69595574494014</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>18.79833936336457</v>
+        <v>18.33759879254464</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.305171469891753</v>
+        <v>0.4565582620914242</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.7872609560339345</v>
+        <v>-3.936865684636677</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6641</v>
+        <v>6546</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>基士德-KY</t>
+          <t>正基</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>307.3953855107001</v>
+        <v>312.9547032703164</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>18.35</v>
+        <v>75</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,16 +3944,16 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>48.33883550074246</v>
+        <v>50.17604797029433</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>18.47475541857973</v>
+        <v>18.79833936336457</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>1.295478810426599</v>
+        <v>0.305171469891753</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.010076981174512</v>
+        <v>-0.7872609560339345</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6561</v>
+        <v>6641</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>是方</t>
+          <t>基士德-KY</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>301.597941943676</v>
+        <v>307.3953855107001</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>338</v>
+        <v>18.35</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>39.95310179169165</v>
+        <v>48.33883550074246</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>15.92831024669716</v>
+        <v>18.47475541857973</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.7831290660455803</v>
+        <v>1.295478810426599</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-2.415889121095163</v>
+        <v>0.010076981174512</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6591</v>
+        <v>6561</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>動力-KY</t>
+          <t>是方</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>297.5295297100117</v>
+        <v>301.597941943676</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>55.5</v>
+        <v>338</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>47.89571698016637</v>
+        <v>39.95310179169165</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>21.27229468791863</v>
+        <v>15.92831024669716</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.3419286435501053</v>
+        <v>0.7831290660455803</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.1213228753602536</v>
+        <v>-2.415889121095163</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6568</v>
+        <v>6591</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>宏觀</t>
+          <t>動力-KY</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>280.2611788583437</v>
+        <v>297.5295297100117</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>176.5</v>
+        <v>55.5</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>36.49207691973459</v>
+        <v>47.89571698016637</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>26.79358854175573</v>
+        <v>21.27229468791863</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.3773273955494983</v>
+        <v>0.3419286435501053</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-2.716731307425485</v>
+        <v>-0.1213228753602536</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6530</v>
+        <v>6568</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>創威</t>
+          <t>宏觀</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>273.3349459004269</v>
+        <v>280.2611788583437</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>97.90000000000001</v>
+        <v>176.5</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,16 +4156,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>43.42085234701366</v>
+        <v>36.49207691973459</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>15.37030248505064</v>
+        <v>26.79358854175573</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.5481834479056017</v>
+        <v>0.3773273955494983</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-1.258141815888457</v>
+        <v>-2.716731307425485</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6624</v>
+        <v>6530</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>萬年清</t>
+          <t>創威</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>264.4797919522783</v>
+        <v>273.3349459004269</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>42.5</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>50.84351011611045</v>
+        <v>43.42085234701366</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>12.87641141601794</v>
+        <v>15.37030248505064</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.1660141506019486</v>
+        <v>0.5481834479056017</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.8466583947305986</v>
+        <v>-1.258141815888457</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, williams_r_recovery, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6689</v>
+        <v>6624</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>伊雲谷</t>
+          <t>萬年清</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>263.0097790658329</v>
+        <v>264.4797919522783</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>67</v>
+        <v>42.5</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,16 +4262,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>43.94801996005704</v>
+        <v>50.84351011611045</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>13.15457280986532</v>
+        <v>12.87641141601794</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.6604450680510734</v>
+        <v>0.1660141506019486</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.2673178463243377</v>
+        <v>-0.8466583947305986</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, williams_r_recovery, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6533</v>
+        <v>6689</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>晶心科</t>
+          <t>伊雲谷</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>237.9493716166865</v>
+        <v>263.0097790658329</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>201.5</v>
+        <v>67</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,16 +4315,16 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>41.54824106436801</v>
+        <v>43.94801996005704</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>17.38626703298286</v>
+        <v>13.15457280986532</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.3659666306626591</v>
+        <v>0.6604450680510734</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-1.991817398688603</v>
+        <v>-0.2673178463243377</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6486</v>
+        <v>6533</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>互動</t>
+          <t>晶心科</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>219.7196600537474</v>
+        <v>237.9493716166865</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>81.8</v>
+        <v>201.5</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>44.91010668425125</v>
+        <v>41.54824106436801</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>17.18046689721345</v>
+        <v>17.38626703298286</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.4919923609059986</v>
+        <v>0.3659666306626591</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>1</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.1066056059074328</v>
+        <v>-1.991817398688603</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6552</v>
+        <v>6486</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>易華電</t>
+          <t>互動</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>193.1053949052276</v>
+        <v>219.7196600537474</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>31.05</v>
+        <v>81.8</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,16 +4421,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>50.2543622094521</v>
+        <v>44.91010668425125</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>16.06653903305078</v>
+        <v>17.18046689721345</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.5920959602831702</v>
+        <v>0.4919923609059986</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.3735132207745319</v>
+        <v>0.1066056059074328</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6577</v>
+        <v>6552</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>勁豐</t>
+          <t>易華電</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>184.5927133941264</v>
+        <v>193.1053949052276</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>75.7</v>
+        <v>31.05</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>32.22666725827857</v>
+        <v>50.2543622094521</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>14.44189594914305</v>
+        <v>16.06653903305078</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>1.359271339412637</v>
+        <v>0.5920959602831702</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.5273502491747291</v>
+        <v>-0.3735132207745319</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6722</v>
+        <v>6577</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>輝創</t>
+          <t>勁豐</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>175.2247126256183</v>
+        <v>184.5927133941264</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>37.4</v>
+        <v>75.7</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>40.84784003316734</v>
+        <v>32.22666725827857</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>15.11452675435338</v>
+        <v>14.44189594914305</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.3261680613668061</v>
+        <v>1.359271339412637</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.1130206901409136</v>
+        <v>-0.5273502491747291</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6835</v>
+        <v>6722</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>圓裕</t>
+          <t>輝創</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>160.2019229840527</v>
+        <v>175.2247126256183</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>36.55</v>
+        <v>37.4</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>42.5552187182104</v>
+        <v>40.84784003316734</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>13.96652691060163</v>
+        <v>15.11452675435338</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.1401610274202643</v>
+        <v>0.3261680613668061</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,62 +4598,115 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.1441846346349169</v>
+        <v>-0.1130206901409136</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
+        <v>6835</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>圓裕</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>160.2019229840527</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>36.55</v>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>42.5552187182104</v>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>13.96652691060163</v>
+      </c>
+      <c r="J79" s="2" t="n">
+        <v>0.1401610274202643</v>
+      </c>
+      <c r="K79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N79" s="2" t="n">
+        <v>-0.1441846346349169</v>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
         <v>6674</v>
       </c>
-      <c r="B79" s="2" t="inlineStr">
+      <c r="B80" s="2" t="inlineStr">
         <is>
           <t>鋐寶科技</t>
         </is>
       </c>
-      <c r="C79" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D79" s="2" t="n">
+      <c r="C80" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D80" s="2" t="n">
         <v>155.3178938175574</v>
       </c>
-      <c r="E79" s="2" t="n">
+      <c r="E80" s="2" t="n">
         <v>17.45</v>
       </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="G79" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H79" s="2" t="n">
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H80" s="2" t="n">
         <v>45.9465259515588</v>
       </c>
-      <c r="I79" s="2" t="n">
+      <c r="I80" s="2" t="n">
         <v>17.1776694624163</v>
       </c>
-      <c r="J79" s="2" t="n">
+      <c r="J80" s="2" t="n">
         <v>0.6990016188308878</v>
       </c>
-      <c r="K79" s="2" t="n">
+      <c r="K80" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M79" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N79" s="2" t="n">
+      <c r="L80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N80" s="2" t="n">
         <v>-0.0056636724478135</v>
       </c>
-      <c r="O79" s="2" t="inlineStr">
+      <c r="O80" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>

</xml_diff>